<commit_message>
Modifying code for reproducability
</commit_message>
<xml_diff>
--- a/histograms/histogram_Alcohol___.xlsx
+++ b/histograms/histogram_Alcohol___.xlsx
@@ -442,79 +442,79 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8.75</v>
+        <v>2.25</v>
       </c>
       <c r="B2" t="n">
-        <v>21917</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>26.25</v>
+        <v>6.75</v>
       </c>
       <c r="B3" t="n">
-        <v>2372</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>43.75</v>
+        <v>11.25</v>
       </c>
       <c r="B4" t="n">
-        <v>698</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>61.25</v>
+        <v>15.75</v>
       </c>
       <c r="B5" t="n">
-        <v>300</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>78.75</v>
+        <v>20.25</v>
       </c>
       <c r="B6" t="n">
-        <v>427</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>96.25</v>
+        <v>24.75</v>
       </c>
       <c r="B7" t="n">
-        <v>338</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>113.75</v>
+        <v>29.25</v>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>131.25</v>
+        <v>33.75</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>148.75</v>
+        <v>38.25</v>
       </c>
       <c r="B10" t="n">
-        <v>239</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>166.25</v>
+        <v>42.75</v>
       </c>
       <c r="B11" t="n">
         <v>0</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>183.75</v>
+        <v>47.25</v>
       </c>
       <c r="B12" t="n">
         <v>0</v>
@@ -530,7 +530,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>201.25</v>
+        <v>51.75</v>
       </c>
       <c r="B13" t="n">
         <v>1</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>218.75</v>
+        <v>56.25</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>236.25</v>
+        <v>60.75</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -554,15 +554,15 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>253.75</v>
+        <v>65.25</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>271.25</v>
+        <v>69.75</v>
       </c>
       <c r="B17" t="n">
         <v>0</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>288.75</v>
+        <v>74.25</v>
       </c>
       <c r="B18" t="n">
         <v>0</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>306.25</v>
+        <v>78.75</v>
       </c>
       <c r="B19" t="n">
         <v>0</v>
@@ -586,7 +586,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>323.75</v>
+        <v>83.25</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
@@ -594,10 +594,10 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>341.25</v>
+        <v>87.75</v>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>